<commit_message>
Update Excel with new results
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -5,17 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{44531D27-F6AB-1143-A1CE-E00DEBD74DF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7115FC4-A1A6-1D46-BF26-AED237407AB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10060" yWindow="1320" windowWidth="20640" windowHeight="16420" activeTab="1" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
     <sheet name="Module 1" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
   <si>
     <t>file</t>
   </si>
@@ -166,132 +165,7 @@
     <t>Nombre d’actes après ajustement pour l’exhaustivité</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Nombre d’actes après correction des anomalies </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>et</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> ajustement pour l’exhaustivité</t>
-    </r>
-  </si>
-  <si>
     <t>Nombre d’actes ajusté (anomalies remplacées par la médiane)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Nombre de rapports </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(établissement × mois)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> soumis</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Nombre de rapports </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(établissement × mois)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> attendus</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Proportion </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(0–1)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> de rapports </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(établissement × mois)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> effectivement soumis</t>
-    </r>
   </si>
   <si>
     <t>Proportion des établissements satisfaisant aux critères de qualité des données</t>
@@ -313,7 +187,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -385,14 +259,6 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -973,7 +839,7 @@
         <v>37</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -990,7 +856,7 @@
         <v>38</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -1007,7 +873,7 @@
         <v>33</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1024,7 +890,7 @@
         <v>32</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -1041,7 +907,7 @@
         <v>31</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -1058,7 +924,7 @@
         <v>30</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1138,144 +1004,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{234E2D60-6B02-084B-BAC6-D9450A049189}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
add details for module 2
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7115FC4-A1A6-1D46-BF26-AED237407AB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FB9C56-5972-DF40-86B5-B809BCB1C1D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10060" yWindow="1320" windowWidth="20640" windowHeight="16420" activeTab="1" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="-32060" yWindow="500" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
     <sheet name="Module 1" sheetId="1" r:id="rId2"/>
+    <sheet name="Module 2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="51">
   <si>
     <t>file</t>
   </si>
@@ -181,6 +182,15 @@
   </si>
   <si>
     <t>Proportion de rapports établissement-mois effectivement soumis</t>
+  </si>
+  <si>
+    <t>control_chart_results.csv</t>
+  </si>
+  <si>
+    <t>count_predict</t>
+  </si>
+  <si>
+    <t>Deseasonalized predicted count, derived using regression-based methods</t>
   </si>
 </sst>
 </file>
@@ -1004,4 +1014,70 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCFDF2BA-F153-AE42-870C-EBFB5A223C41}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" customWidth="1"/>
+    <col min="4" max="4" width="45.33203125" customWidth="1"/>
+    <col min="5" max="5" width="62.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add details for output_consistency
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FB9C56-5972-DF40-86B5-B809BCB1C1D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E5E443A-A650-AD4E-92DC-D709F3FDCF2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-32060" yWindow="500" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="-37440" yWindow="-7680" windowWidth="37440" windowHeight="21100" activeTab="1" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="61">
   <si>
     <t>file</t>
   </si>
@@ -191,13 +191,43 @@
   </si>
   <si>
     <t>Deseasonalized predicted count, derived using regression-based methods</t>
+  </si>
+  <si>
+    <t>output_consistency.csv</t>
+  </si>
+  <si>
+    <t>consistency_ratio</t>
+  </si>
+  <si>
+    <t>sconsistency</t>
+  </si>
+  <si>
+    <t>ratio_type</t>
+  </si>
+  <si>
+    <t>Type of ratio being assessed</t>
+  </si>
+  <si>
+    <t>Type de ratio évalué</t>
+  </si>
+  <si>
+    <t>Calculated ratio for inter-indicator consistency evaluation</t>
+  </si>
+  <si>
+    <t>Ratio calculé pour l'évaluation de la cohérence inter-indicateurs</t>
+  </si>
+  <si>
+    <t>Binary variable indicating whether the ratio meets consistency criteria (1 = meets, 0 = does not meet)</t>
+  </si>
+  <si>
+    <t>Variable binaire indiquant si le ratio respecte les critères de cohérence (1 = respecte, 0 = ne respecte pas)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -241,12 +271,6 @@
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -308,21 +332,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -756,7 +779,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57657D03-3711-F742-855B-C85A7C1EAEEF}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
@@ -785,230 +808,272 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="9" t="s">
+      <c r="C2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="C3" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="9" t="s">
+      <c r="C4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="C5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="10" t="s">
+      <c r="C6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="9" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="9" t="s">
+      <c r="C8" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="C9" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="10" t="s">
+      <c r="C10" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="9" t="s">
         <v>43</v>
       </c>
     </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B12" s="6"/>
-    </row>
-    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
+      <c r="A12" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
       <c r="C14"/>
-      <c r="D14"/>
       <c r="E14"/>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
       <c r="C15"/>
-      <c r="D15"/>
       <c r="E15"/>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
     </row>
-    <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
+    <row r="17" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17"/>
     </row>
-    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
+    <row r="18" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
       <c r="C18"/>
       <c r="D18"/>
       <c r="E18"/>
     </row>
-    <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
       <c r="C19"/>
       <c r="D19"/>
       <c r="E19"/>
     </row>
-    <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
+    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
       <c r="C20"/>
       <c r="D20"/>
       <c r="E20"/>
     </row>
-    <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
       <c r="C21"/>
       <c r="D21"/>
       <c r="E21"/>
     </row>
-    <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
       <c r="C22"/>
       <c r="D22"/>
       <c r="E22"/>
+    </row>
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="G24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1046,36 +1111,36 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="9" t="s">
+      <c r="C2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="C3" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="E3" s="9"/>
+      <c r="E3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated file names and added the top outlier output
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DF73F00-5C17-2745-8AAB-FE482EE205A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313BE865-468E-E944-ADE2-6E51391C556B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4800" yWindow="2300" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="69">
   <si>
     <t>file</t>
   </si>
@@ -104,9 +104,6 @@
     <t>time</t>
   </si>
   <si>
-    <t>output_outliers.csv</t>
-  </si>
-  <si>
     <t>count_adjust</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>completeness_percentage</t>
   </si>
   <si>
-    <t>completeness_long_format.csv</t>
-  </si>
-  <si>
     <t>Proportion of facility-month reports actually submitted</t>
   </si>
   <si>
@@ -209,15 +203,6 @@
     <t>Variable binaire indiquant si le ratio respecte les critères de cohérence (1 = respecte, 0 = ne respecte pas)</t>
   </si>
   <si>
-    <t>output_consistency_geo.csv</t>
-  </si>
-  <si>
-    <t>output_consistency_facility.csv</t>
-  </si>
-  <si>
-    <t>facility_dqa.csv</t>
-  </si>
-  <si>
     <t>dqa_temp</t>
   </si>
   <si>
@@ -225,6 +210,42 @@
   </si>
   <si>
     <t>Variable binaire indiquant si l'établissement répond aux critères de l'évaluation DQA (1 = répond, 0 = ne répond pas).</t>
+  </si>
+  <si>
+    <t>M1_output_outliers.csv</t>
+  </si>
+  <si>
+    <t>M1_completeness_long_format.csv</t>
+  </si>
+  <si>
+    <t>M1_facility_dqa.csv</t>
+  </si>
+  <si>
+    <t>M1_output_consistency_geo.csv</t>
+  </si>
+  <si>
+    <t>M1_output_consistency_facility.csv</t>
+  </si>
+  <si>
+    <t>M1_top_outliers_data.csv</t>
+  </si>
+  <si>
+    <t>max_percent_change</t>
+  </si>
+  <si>
+    <t>mean_volIM</t>
+  </si>
+  <si>
+    <t>Maximum percentage change due to outlier adjustment</t>
+  </si>
+  <si>
+    <t>Average volume after outlier adjustmen</t>
+  </si>
+  <si>
+    <t>Changement maximal en pourcentage entre les valeurs ajustées et originales</t>
+  </si>
+  <si>
+    <t>Volume moyen après ajustement des anomalies</t>
   </si>
 </sst>
 </file>
@@ -701,7 +722,7 @@
     </row>
     <row r="2" spans="1:2" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>8</v>
@@ -813,204 +834,224 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>22</v>
-      </c>
       <c r="C2" s="9" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>29</v>
-      </c>
       <c r="E4" s="8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>28</v>
-      </c>
       <c r="E5" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>19</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13"/>
-      <c r="D13"/>
-      <c r="E13"/>
-    </row>
-    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14"/>
-      <c r="D14"/>
-      <c r="E14"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="12"/>
@@ -1089,10 +1130,10 @@
         <v>8</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1106,10 +1147,10 @@
         <v>8</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1123,10 +1164,10 @@
         <v>8</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -1140,10 +1181,10 @@
         <v>8</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1182,33 +1223,33 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>44</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>46</v>
       </c>
       <c r="E3" s="8"/>
     </row>

</xml_diff>

<commit_message>
added module 4 results
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75458CC8-8660-B746-AAFE-6BCD6A6EE117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940DBD13-C116-1646-BB2A-624AB8A58E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="920" yWindow="500" windowWidth="27880" windowHeight="17500" activeTab="2" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="840" yWindow="500" windowWidth="27880" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
     <sheet name="Module 1 (dqa)" sheetId="1" r:id="rId2"/>
     <sheet name="Module 2 (adjustments)" sheetId="4" r:id="rId3"/>
     <sheet name="Module 3 (control chart)" sheetId="3" r:id="rId4"/>
+    <sheet name="Module 4 (coverage estimate)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="60">
   <si>
     <t>file</t>
   </si>
@@ -204,6 +205,21 @@
   </si>
   <si>
     <t>outlier_flag</t>
+  </si>
+  <si>
+    <t>M4_Coverage_estimation.csv</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>coverage</t>
+  </si>
+  <si>
+    <t>estimated coverage</t>
+  </si>
+  <si>
+    <t>"official_estimate" = Official estimate; "avgsurveyprojection" =  Extrapolated estimates ; "count" =  HMIS annual volume  ; "cov" = HMIS estimates</t>
   </si>
 </sst>
 </file>
@@ -1058,4 +1074,67 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31BD6EA-B880-1641-87C8-784E246E1427}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="4" max="4" width="101.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="8"/>
+      <c r="F2" s="6"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="8"/>
+      <c r="F3" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
pivot results to wide, results updated
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940DBD13-C116-1646-BB2A-624AB8A58E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DE88D9-F6CF-E540-AA9D-993C34F8AEC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="500" windowWidth="27880" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="1060" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="64">
   <si>
     <t>file</t>
   </si>
@@ -210,16 +210,28 @@
     <t>M4_Coverage_estimation.csv</t>
   </si>
   <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>coverage</t>
-  </si>
-  <si>
-    <t>estimated coverage</t>
-  </si>
-  <si>
-    <t>"official_estimate" = Official estimate; "avgsurveyprojection" =  Extrapolated estimates ; "count" =  HMIS annual volume  ; "cov" = HMIS estimates</t>
+    <t>coverage_official_estimate</t>
+  </si>
+  <si>
+    <t>coverage_cov</t>
+  </si>
+  <si>
+    <t>coverage_avgsurveyprojection</t>
+  </si>
+  <si>
+    <t>Official estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coverage_count     </t>
+  </si>
+  <si>
+    <t>HMIS annual volume</t>
+  </si>
+  <si>
+    <t>HMIS estimates</t>
+  </si>
+  <si>
+    <t>Extrapolated estimates</t>
   </si>
 </sst>
 </file>
@@ -1078,14 +1090,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31BD6EA-B880-1641-87C8-784E246E1427}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
-    <col min="4" max="4" width="101.33203125" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1102,7 +1115,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>55</v>
       </c>
@@ -1110,29 +1123,57 @@
         <v>56</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>59</v>
       </c>
       <c r="E2" s="8"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="8"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="8"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="6"/>
+      <c r="C5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
removed unnecessary columns from output - updated results object file
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B4E25D-1260-8042-98DD-4126D4F3C777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6E1CCD-C95B-6344-A71B-AABEC2616311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="6500" yWindow="8520" windowWidth="27740" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="63">
   <si>
     <t>file</t>
   </si>
@@ -208,12 +208,6 @@
   </si>
   <si>
     <t>coverage_avgsurveyprojection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coverage_count     </t>
-  </si>
-  <si>
-    <t>HMIS annual volume</t>
   </si>
   <si>
     <t>HMIS estimates</t>
@@ -980,10 +974,10 @@
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1014,7 +1008,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>26</v>
@@ -1065,10 +1059,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1093,7 +1087,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31BD6EA-B880-1641-87C8-784E246E1427}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
@@ -1129,7 +1123,7 @@
         <v>7</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E2" s="8"/>
     </row>
@@ -1144,7 +1138,7 @@
         <v>7</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E3" s="8"/>
     </row>
@@ -1153,30 +1147,15 @@
         <v>52</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="E4" s="8"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated outputs from M2, added value in M1 (DQA mean)
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6E1CCD-C95B-6344-A71B-AABEC2616311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8EB2C22-57D8-4B44-8AD1-6C1C5C35C732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6500" yWindow="8520" windowWidth="27740" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="7860" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="2" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="67">
   <si>
     <t>file</t>
   </si>
@@ -229,6 +229,18 @@
   </si>
   <si>
     <t>Official estimates</t>
+  </si>
+  <si>
+    <t>M2_adjusted_data_admin_area.csv</t>
+  </si>
+  <si>
+    <t>M2_adjusted_data_national.csv</t>
+  </si>
+  <si>
+    <t>dqa_mean</t>
+  </si>
+  <si>
+    <t>Mean DQA score: overall measure of data quality compliance</t>
   </si>
 </sst>
 </file>
@@ -300,7 +312,7 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -319,6 +331,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -332,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -345,6 +363,9 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -778,7 +799,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57657D03-3711-F742-855B-C85A7C1EAEEF}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
@@ -858,37 +879,35 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>34</v>
-      </c>
+      <c r="A5" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="9"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>44</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -896,20 +915,37 @@
         <v>44</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="C8" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="7:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="G24"/>
+    <row r="25" spans="7:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="G25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -919,7 +955,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80212091-6541-4E49-8496-BDDBD6A354D7}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" customWidth="1"/>
@@ -1011,6 +1047,142 @@
         <v>59</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated module 1, 2, 3
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8EB2C22-57D8-4B44-8AD1-6C1C5C35C732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844F1F41-C1D7-BE4F-8A94-A85E471057F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7860" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="2" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="7860" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="1" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
     <sheet name="Module 1 (dqa)" sheetId="1" r:id="rId2"/>
     <sheet name="Module 2 (adjustments)" sheetId="4" r:id="rId3"/>
-    <sheet name="Module 3 (control chart)" sheetId="3" r:id="rId4"/>
+    <sheet name="Module 3 (service utilization)" sheetId="3" r:id="rId4"/>
     <sheet name="Module 4 (coverage estimate)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="68">
   <si>
     <t>file</t>
   </si>
@@ -102,9 +102,6 @@
     <t>time</t>
   </si>
   <si>
-    <t>count_adjust</t>
-  </si>
-  <si>
     <t>count</t>
   </si>
   <si>
@@ -123,15 +120,6 @@
     <t>Nombre d’actes après correction des anomalies et ajustement pour l’exhaustivité</t>
   </si>
   <si>
-    <t>control_chart_results.csv</t>
-  </si>
-  <si>
-    <t>count_predict</t>
-  </si>
-  <si>
-    <t>Deseasonalized predicted count, derived using regression-based methods</t>
-  </si>
-  <si>
     <t>consistency_ratio</t>
   </si>
   <si>
@@ -222,9 +210,6 @@
     <t>Number of services after both outlier and completeness adjustment</t>
   </si>
   <si>
-    <t>Number of services after outlier adjustment</t>
-  </si>
-  <si>
     <t>Nombre d’actes après correction des anomalies</t>
   </si>
   <si>
@@ -241,6 +226,24 @@
   </si>
   <si>
     <t>Mean DQA score: overall measure of data quality compliance</t>
+  </si>
+  <si>
+    <t>M3_service_utilization.csv</t>
+  </si>
+  <si>
+    <t>M3_disruptions_analysis.csv</t>
+  </si>
+  <si>
+    <t>expect_national</t>
+  </si>
+  <si>
+    <t>expect_province</t>
+  </si>
+  <si>
+    <t>Expected service utilization (national trend-adjusted)</t>
+  </si>
+  <si>
+    <t>Expected service utilization (province trend-adjusted)</t>
   </si>
 </sst>
 </file>
@@ -717,7 +720,7 @@
     </row>
     <row r="2" spans="1:2" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>7</v>
@@ -829,119 +832,119 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="E2" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>46</v>
-      </c>
       <c r="E3" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E5" s="9"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="7:7" ht="16" x14ac:dyDescent="0.2">
@@ -984,7 +987,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>3</v>
@@ -993,15 +996,15 @@
         <v>7</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>4</v>
@@ -1010,15 +1013,15 @@
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>5</v>
@@ -1027,15 +1030,15 @@
         <v>7</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>6</v>
@@ -1044,15 +1047,15 @@
         <v>7</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>3</v>
@@ -1061,15 +1064,15 @@
         <v>7</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>4</v>
@@ -1078,15 +1081,15 @@
         <v>7</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>5</v>
@@ -1095,15 +1098,15 @@
         <v>7</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>6</v>
@@ -1112,15 +1115,15 @@
         <v>7</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>3</v>
@@ -1129,15 +1132,15 @@
         <v>7</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>4</v>
@@ -1146,15 +1149,15 @@
         <v>7</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>5</v>
@@ -1163,15 +1166,15 @@
         <v>7</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>6</v>
@@ -1180,10 +1183,10 @@
         <v>7</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1193,10 +1196,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCFDF2BA-F153-AE42-870C-EBFB5A223C41}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="19.1640625" customWidth="1"/>
     <col min="3" max="3" width="12.1640625" customWidth="1"/>
     <col min="4" max="4" width="45.33203125" customWidth="1"/>
@@ -1222,35 +1225,101 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="8"/>
+        <v>54</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6" s="14"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1286,46 +1355,46 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>56</v>
       </c>
       <c r="E4" s="8"/>
     </row>

</xml_diff>

<commit_message>
remove 2024 from surveys - carry back extrapolated estimates
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844F1F41-C1D7-BE4F-8A94-A85E471057F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF17EDAA-5D12-B049-8ECE-AD8B13C2A3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7860" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="1" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="7860" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="3" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
@@ -180,9 +180,6 @@
     <t>M2_adjusted_data.csv</t>
   </si>
   <si>
-    <t>completeness_lag</t>
-  </si>
-  <si>
     <t>outlier_flag</t>
   </si>
   <si>
@@ -244,6 +241,9 @@
   </si>
   <si>
     <t>Expected service utilization (province trend-adjusted)</t>
+  </si>
+  <si>
+    <t>completeness_flag</t>
   </si>
 </sst>
 </file>
@@ -835,7 +835,7 @@
         <v>37</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>7</v>
@@ -852,7 +852,7 @@
         <v>38</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
@@ -886,13 +886,13 @@
         <v>39</v>
       </c>
       <c r="B5" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>61</v>
       </c>
       <c r="E5" s="9"/>
     </row>
@@ -1013,10 +1013,10 @@
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1047,7 +1047,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>25</v>
@@ -1055,7 +1055,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>3</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>4</v>
@@ -1081,15 +1081,15 @@
         <v>7</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>5</v>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>6</v>
@@ -1115,7 +1115,7 @@
         <v>7</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>25</v>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>3</v>
@@ -1140,7 +1140,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>4</v>
@@ -1149,15 +1149,15 @@
         <v>7</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>5</v>
@@ -1174,7 +1174,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>6</v>
@@ -1183,7 +1183,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>25</v>
@@ -1225,7 +1225,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>3</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>4</v>
@@ -1251,15 +1251,15 @@
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>5</v>
@@ -1276,7 +1276,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>6</v>
@@ -1285,7 +1285,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>25</v>
@@ -1293,31 +1293,31 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>64</v>
-      </c>
       <c r="C6" s="14" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E7" s="14"/>
     </row>
@@ -1355,46 +1355,46 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>49</v>
-      </c>
       <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E4" s="8"/>
     </row>

</xml_diff>

<commit_message>
add detail re new output in M4 - result file
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{823B02AA-23F5-F244-8309-B8CB88E32147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907AB164-9E4D-3E49-B03F-E16E37A5F132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7860" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="73">
   <si>
     <t>file</t>
   </si>
@@ -183,9 +183,6 @@
     <t>outlier_flag</t>
   </si>
   <si>
-    <t>M4_Coverage_estimation.csv</t>
-  </si>
-  <si>
     <t>coverage_official_estimate</t>
   </si>
   <si>
@@ -256,6 +253,12 @@
   </si>
   <si>
     <t xml:space="preserve">Rank of best (1) to worse (3 or 4) denominator </t>
+  </si>
+  <si>
+    <t>M4_coverage_estimation_admin_area_2</t>
+  </si>
+  <si>
+    <t>M4_coverage_estimation.csv</t>
   </si>
 </sst>
 </file>
@@ -365,7 +368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -381,9 +384,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -867,7 +867,7 @@
         <v>38</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
@@ -901,13 +901,13 @@
         <v>39</v>
       </c>
       <c r="B5" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>60</v>
       </c>
       <c r="E5" s="9"/>
     </row>
@@ -1028,10 +1028,10 @@
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1062,7 +1062,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>25</v>
@@ -1070,7 +1070,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>3</v>
@@ -1087,7 +1087,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>4</v>
@@ -1096,15 +1096,15 @@
         <v>7</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>5</v>
@@ -1121,7 +1121,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>6</v>
@@ -1130,7 +1130,7 @@
         <v>7</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>25</v>
@@ -1138,7 +1138,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>3</v>
@@ -1155,7 +1155,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>4</v>
@@ -1164,15 +1164,15 @@
         <v>7</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>5</v>
@@ -1189,7 +1189,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>6</v>
@@ -1198,7 +1198,7 @@
         <v>7</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>25</v>
@@ -1240,7 +1240,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>3</v>
@@ -1257,7 +1257,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>4</v>
@@ -1266,15 +1266,15 @@
         <v>7</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>5</v>
@@ -1291,7 +1291,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>6</v>
@@ -1300,7 +1300,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>25</v>
@@ -1308,31 +1308,31 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>63</v>
-      </c>
       <c r="C6" s="14" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E7" s="14"/>
     </row>
@@ -1343,12 +1343,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B31BD6EA-B880-1641-87C8-784E246E1427}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
     <col min="2" max="2" width="27.6640625" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -1370,79 +1370,90 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>48</v>
-      </c>
       <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E4" s="8"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="15"/>
+      <c r="B7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>50</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated the disruption analysis with results aggregated and parameter to set threshold for diff between actual and predicted
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907AB164-9E4D-3E49-B03F-E16E37A5F132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BF0D81-6160-4D4C-9A4B-272AFA5FFC05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7860" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="4" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="780" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="3" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Module 3 (service utilization)" sheetId="3" r:id="rId4"/>
     <sheet name="Module 4 (coverage estimate)" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="76">
   <si>
     <t>file</t>
   </si>
@@ -225,21 +225,6 @@
     <t>M3_service_utilization.csv</t>
   </si>
   <si>
-    <t>M3_disruptions_analysis.csv</t>
-  </si>
-  <si>
-    <t>expect_national</t>
-  </si>
-  <si>
-    <t>expect_province</t>
-  </si>
-  <si>
-    <t>Expected service utilization (national trend-adjusted)</t>
-  </si>
-  <si>
-    <t>Expected service utilization (province trend-adjusted)</t>
-  </si>
-  <si>
     <t>completeness_flag</t>
   </si>
   <si>
@@ -259,6 +244,30 @@
   </si>
   <si>
     <t>M4_coverage_estimation.csv</t>
+  </si>
+  <si>
+    <t>M3_disruptions_analysis_admin_area_1.csv</t>
+  </si>
+  <si>
+    <t>count_expect_diff</t>
+  </si>
+  <si>
+    <t>M3_disruptions_analysis_admin_area_2.csv</t>
+  </si>
+  <si>
+    <t>diff_percent</t>
+  </si>
+  <si>
+    <t>Percent difference between actual and predicted volume</t>
+  </si>
+  <si>
+    <t>Expected services when difference exceeds threshold; otherwise reported value</t>
+  </si>
+  <si>
+    <t>Écart en pourcentage entre le volume observé et le volume attendu</t>
+  </si>
+  <si>
+    <t>Volume attendu si l’écart dépasse le seuil ; sinon, valeur observée</t>
   </si>
 </sst>
 </file>
@@ -867,7 +876,7 @@
         <v>38</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>7</v>
@@ -1211,10 +1220,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCFDF2BA-F153-AE42-870C-EBFB5A223C41}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="1" max="1" width="42.6640625" customWidth="1"/>
     <col min="2" max="2" width="19.1640625" customWidth="1"/>
     <col min="3" max="3" width="12.1640625" customWidth="1"/>
     <col min="4" max="4" width="45.33203125" customWidth="1"/>
@@ -1308,33 +1317,103 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="14"/>
+        <v>21</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E7" s="14"/>
+        <v>72</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>75</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1370,7 +1449,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>47</v>
@@ -1385,7 +1464,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>49</v>
@@ -1400,7 +1479,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>48</v>
@@ -1415,35 +1494,35 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
added output for regression with random effet at admin_area_3
</commit_message>
<xml_diff>
--- a/Results object details.xlsx
+++ b/Results object details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claireboulange/Desktop/FASTR/R codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BF0D81-6160-4D4C-9A4B-272AFA5FFC05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFC6B36-E8AB-F546-831F-F90C443BCE5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="3" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
+    <workbookView xWindow="1000" yWindow="500" windowWidth="27740" windowHeight="17500" activeTab="3" xr2:uid="{375A38BE-D388-CF4E-8910-AD552D2DCFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="DEFAULTS" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="77">
   <si>
     <t>file</t>
   </si>
@@ -268,6 +268,9 @@
   </si>
   <si>
     <t>Volume attendu si l’écart dépasse le seuil ; sinon, valeur observée</t>
+  </si>
+  <si>
+    <t>M3_disruptions_analysis_admin_area_3.csv</t>
   </si>
 </sst>
 </file>
@@ -1220,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCFDF2BA-F153-AE42-870C-EBFB5A223C41}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42.6640625" customWidth="1"/>
@@ -1412,6 +1415,57 @@
         <v>73</v>
       </c>
       <c r="E11" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="14" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>